<commit_message>
This is Updated File in which thier is information about the Data Engineer
</commit_message>
<xml_diff>
--- a/Second bit of transition.xlsx
+++ b/Second bit of transition.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\OneDrive\Desktop\Data Engineer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E8FDCE-D2F9-40DB-BD71-B769DA0B52B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F6D6B47-4EED-47AF-8710-598ADCAE3D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Bit 2 — Learn Data Engineering Tools</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t>Logs → BigQuery pipeline</t>
+  </si>
+  <si>
+    <t>…</t>
   </si>
 </sst>
 </file>
@@ -409,61 +412,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>9</v>
       </c>

</xml_diff>